<commit_message>
chore: Excel güncelle (saha_durum_operasyon_tablosu.xlsx) — dashboard üzerinden gönderildi
</commit_message>
<xml_diff>
--- a/saha_durum_operasyon_tablosu.xlsx
+++ b/saha_durum_operasyon_tablosu.xlsx
@@ -1,33 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acevizci\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sdursun\Desktop\YÖNETİM PROJE TAKİP RAPOR\02.1 Ağustos 2026 Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65413923-3649-4549-B2F1-8E5EDEAA9837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3B9422-3A13-43B5-B53E-78BFA59DC929}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13920" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Saha Durum" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -583,10 +572,10 @@
         <v>94</v>
       </c>
       <c r="B4" s="2">
-        <v>1713</v>
+        <v>1703</v>
       </c>
       <c r="C4" s="2">
-        <v>1612</v>
+        <v>1638</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -602,7 +591,7 @@
     </row>
     <row r="7" spans="1:5" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7" s="2">
         <v>937</v>
@@ -650,13 +639,13 @@
         <v>14</v>
       </c>
       <c r="B12" s="4">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C12" s="4">
-        <v>523</v>
+        <v>459</v>
       </c>
       <c r="D12" s="4">
-        <v>540</v>
+        <v>474</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>15</v>
@@ -684,13 +673,13 @@
         <v>19</v>
       </c>
       <c r="B14" s="4">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C14" s="4">
-        <v>955</v>
+        <v>803</v>
       </c>
       <c r="D14" s="4">
-        <v>985</v>
+        <v>827</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>20</v>
@@ -701,13 +690,13 @@
         <v>21</v>
       </c>
       <c r="B15" s="4">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C15" s="4">
-        <v>261</v>
+        <v>397</v>
       </c>
       <c r="D15" s="4">
-        <v>269</v>
+        <v>412</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>22</v>
@@ -718,13 +707,13 @@
         <v>23</v>
       </c>
       <c r="B16" s="4">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C16" s="4">
-        <v>950</v>
+        <v>974</v>
       </c>
       <c r="D16" s="4">
-        <v>976</v>
+        <v>1001</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>24</v>
@@ -752,13 +741,13 @@
         <v>27</v>
       </c>
       <c r="B18" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C18" s="4">
-        <v>138</v>
+        <v>194</v>
       </c>
       <c r="D18" s="4">
-        <v>143</v>
+        <v>200</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>28</v>
@@ -770,7 +759,7 @@
       </c>
       <c r="B19" s="7">
         <f>SUM(B11:B18)</f>
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C19" s="7">
         <f>SUM(C11:C18)</f>
@@ -778,7 +767,7 @@
       </c>
       <c r="D19" s="7">
         <f>SUM(D11:D18)</f>
-        <v>2999</v>
+        <v>3000</v>
       </c>
       <c r="E19" s="8" t="s">
         <v>30</v>
@@ -794,6 +783,233 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="de48f57a-7a98-42ae-8400-a2fbfcb9b9a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EB4C2675C53E6A4DB1D8BC8AD034CCC1" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="604af05efb6f7a4fa4d9b65a9922e243">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="de48f57a-7a98-42ae-8400-a2fbfcb9b9a5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0386dbcb163751ea84dc3c1f3a1ba8df" ns2:_="">
+    <xsd:import namespace="de48f57a-7a98-42ae-8400-a2fbfcb9b9a5"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="de48f57a-7a98-42ae-8400-a2fbfcb9b9a5" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7b1e589d-88e8-49d4-851b-d1cb70381577" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="14" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90551FEF-EEB5-4761-9E89-2DE4B617EEEF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="de48f57a-7a98-42ae-8400-a2fbfcb9b9a5"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F8AA350-7ECB-412F-AC7B-16317C5370E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB51F81E-0EA4-4AE0-BD9A-239FA574BD6B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="de48f57a-7a98-42ae-8400-a2fbfcb9b9a5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>